<commit_message>
Ticket 18: triage the source data findings; full GLEIF runs no longer block on invalid LEIs
Triage (operator agreed, 2026-09-29), each finding checked against main
and the data: accept 1 (with a guard) and 2a; 2b has 0 records in scope,
so nothing to fix; fix 3 here; keep 4 as fog; fix 5 and 6 next.

- GLEIF contracts: invalid_lei and invalid_lei_checksum are non-blocking.
  The Company scope passes the lei format when a release is validated, so an
  invalid LEI can never be ours; 356 such records blocked every full run.
  New contract digests are pinned, the earlier ones still peelable.
- record_evidence refuses a record whose gleif:Deletion holds a value
  (blocking): GLEIF flags deletions in delta files only, and a delta release
  is accepted. The 257,509 empty flags in the full file read as before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V75sGum1vG9w3NFXJLh4XQ
</commit_message>
<xml_diff>
--- a/rules/sources/gleif/MAPPING.xlsx
+++ b/rules/sources/gleif/MAPPING.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>outside_approved_company_scope, unsupported_identity_kind, reported_parent_exception, quality_name_present</t>
+          <t>outside_approved_company_scope, unsupported_identity_kind, reported_parent_exception, invalid_lei, invalid_lei_checksum, quality_name_present</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>outside_approved_company_scope, unsupported_identity_kind, reported_parent_exception</t>
+          <t>outside_approved_company_scope, unsupported_identity_kind, reported_parent_exception, invalid_lei, invalid_lei_checksum</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>outside_approved_company_scope, unsupported_identity_kind, reported_parent_exception</t>
+          <t>outside_approved_company_scope, unsupported_identity_kind, reported_parent_exception, invalid_lei, invalid_lei_checksum</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GLEIF's successor entity, read from its lists (profiling 04c)
- Contract language: a relationship mapping may read lists. `each` makes
  one link per item (paths `item.`); `find` adds the first item of another
  list whose `where` paths match (any element of a nested list), read
  under its name. Mappings without them read as before.
- rules/sources/gleif/source.yaml, gleif.level1.v1: SUCCESSOR_ENTITY per
  successor LEI, dated by the completed event naming it, with the event
  type and status. GLEIF Level 1 contract c7655ed6..., peel back to
  74b8b1f4....
- Mapping Document lists each/find; REFERENCE.md says them.
- PG16: a GLEIF successor ends the child's parent link and its calculated
  ultimate parent on the event date.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A3rb2CVqe8oyC2exiUCb51
</commit_message>
<xml_diff>
--- a/rules/sources/gleif/MAPPING.xlsx
+++ b/rules/sources/gleif/MAPPING.xlsx
@@ -710,14 +710,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1560,62 +1560,158 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>gleif.relationships.v1</t>
+          <t>gleif.level1.v1</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>relationship IS_DIRECTLY_CONSOLIDATED_BY, IS_ULTIMATELY_CONSOLIDATED_BY</t>
+          <t>relationship SUCCESSOR_ENTITY</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>from</t>
+          <t>to</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>start</t>
+          <t>item.SuccessorLEI.$</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Link from gleif.level1.v1</t>
+          <t>Link to gleif.level1.v1</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.relationships.v1.contract.adapter.relationships</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.relationships</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>relationship SUCCESSOR_ENTITY</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Entity.SuccessorEntity</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>One link per item (item.)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>mdm.gleif.level1.v1.contract.adapter.relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>relationship SUCCESSOR_ENTITY</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Entity.LegalEntityEvents.LegalEntityEvent</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>The first item where @event_status = COMPLETED; AffectedFields.AffectedField.$ = item.SuccessorLEI.$ (event.)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>mdm.gleif.level1.v1.contract.adapter.relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>gleif.relationships.v1</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>relationship IS_DIRECTLY_CONSOLIDATED_BY, IS_ULTIMATELY_CONSOLIDATED_BY</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Link from gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>mdm.gleif.relationships.v1.contract.adapter.relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>gleif.relationships.v1</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>relationship IS_DIRECTLY_CONSOLIDATED_BY, IS_ULTIMATELY_CONSOLIDATED_BY</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>to</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>end</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Link to gleif.level1.v1</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>mdm.gleif.relationships.v1.contract.adapter.relationships</t>
         </is>

</xml_diff>

<commit_message>
L6: a non-object GLEIF Extension fails closed; the rulings recorded
The operator, 2026-10-10 17:55 ET: "approve both digests, go with your
recommendations". Relationships 78cb4dd5... and reporting exceptions
8ec18c6d... approved on the whole-file evidence. Out-of-scope records:
dropped by the reading (policy-language spec updated). A non-object
Extension is read as the deletion flag itself, as the older reader did:
new digests 67fe1aaa..., b9b1fd11..., 643e8335..., each peeling to the
approved one, await approval. MAPPING.xlsx regenerated from the rules.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFKdv4nqKXKM9d5Cf2hEFk
</commit_message>
<xml_diff>
--- a/rules/sources/gleif/MAPPING.xlsx
+++ b/rules/sources/gleif/MAPPING.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>start</t>
+          <t>RelationshipRecord.Relationship.StartNode.NodeID.$</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>end</t>
+          <t>RelationshipRecord.Relationship.EndNode.NodeID.$</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1712,6 +1712,38 @@
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>mdm.gleif.relationships.v1.contract.adapter.relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>gleif.relationships.v1</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>relationship IS_DIRECTLY_CONSOLIDATED_BY, IS_ULTIMATELY_CONSOLIDATED_BY</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>period</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>RelationshipRecord.Relationship.RelationshipPeriods.RelationshipPeriod</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>The first item where PeriodType.$ = RELATIONSHIP_PERIOD (period.)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>mdm.gleif.relationships.v1.contract.adapter.relationships</t>
         </is>

</xml_diff>

<commit_message>
Issue 20 L7: the reading is a contract's one statement of its fields
The hand-written record mapping in adapters.py is gone: a record's fields
and matching values come only from the contract's reading. ADV's two
contracts get readings (all 13 local months equal record for record under
the old mapping first); the older fields, matching and field_shape lists
leave all four sources' contracts and registration refuses them. The
workbook and the catalog read each field's path from the reading. Tests
that compared the reading with the old mapping now check what it gave,
taken from it on main.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rules/sources/gleif/MAPPING.xlsx
+++ b/rules/sources/gleif/MAPPING.xlsx
@@ -777,7 +777,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.name</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.name</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.address</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.jurisdiction</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.jurisdiction</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_legal_form</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_legal_form</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_entity_status</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_entity_status</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_registration_status</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_registration_status</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_initial_registration</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_initial_registration</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_last_update</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_last_update</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_next_renewal</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_next_renewal</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_managing_lou</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_managing_lou</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_validation_source</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_validation_source</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_registration_authority</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_registration_authority</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_registration_authority_entity_id</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_registration_authority_entity_id</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.fields.gleif_entity_creation_date</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.gleif_entity_creation_date</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.matching.headquarters_postal_code</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.matching.object.fields.headquarters_postal_code</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.matching.headquarters_country</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.matching.object.fields.headquarters_country</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.matching.headquarters_address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.matching.object.fields.headquarters_address</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.matching.headquarters_address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.matching.object.fields.headquarters_address</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.matching.headquarters_address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.matching.object.fields.headquarters_address</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.matching.headquarters_address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.matching.object.fields.headquarters_address</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.matching.headquarters_address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.matching.object.fields.headquarters_address</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>mdm.gleif.level1.v1.contract.adapter.matching.headquarters_address</t>
+          <t>mdm.gleif.level1.v1.contract.adapter.reading.read.tables.mapped.columns.matching.object.fields.headquarters_address</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticket 10, part 1: the Person and link checks, both Person feeds
The checks the operator approved on 2026-10-02 ("Proposed set"):
- the name holds a letter (pattern@1, quality v2 in both feeds);
- a bad or missing CIK sets the record aside without stopping the run;
- `ends: {reason}`, a new opt-in link rule: a record whose link names no
  end is set aside instead of losing the link silently;
- `interval: {reason}` on the three insider links (no date: set aside);
- a test holds every contract's capacities to its type's list.
Every new reason is non-blocking. The Mapping Document shows each link's
rules; REFERENCE.md documents them. Measured first on the local copies
(counts only): nothing is set aside today.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AoWChUCsVyST73AjRcdH6D
</commit_message>
<xml_diff>
--- a/rules/sources/gleif/MAPPING.xlsx
+++ b/rules/sources/gleif/MAPPING.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1730,20 +1730,84 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
+          <t>interval</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>invalid_relationship_interval</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Sets the record aside when the link has no start, or ends before it starts</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>mdm.gleif.relationships.v1.contract.adapter.relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>gleif.relationships.v1</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>relationship IS_DIRECTLY_CONSOLIDATED_BY, IS_ULTIMATELY_CONSOLIDATED_BY</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>invalid_relationship_status_interval</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Sets the record aside when the status is not allowed, or needs an end it lacks</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>mdm.gleif.relationships.v1.contract.adapter.relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>gleif.relationships.v1</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>relationship IS_DIRECTLY_CONSOLIDATED_BY, IS_ULTIMATELY_CONSOLIDATED_BY</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
           <t>period</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>RelationshipRecord.Relationship.RelationshipPeriods.RelationshipPeriod</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>The first item where PeriodType.$ = RELATIONSHIP_PERIOD (period.)</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>mdm.gleif.relationships.v1.contract.adapter.relationships</t>
         </is>

</xml_diff>

<commit_message>
Cover configured entities and pipelines in the rules catalog
Generate all source/pipeline/relationship workbooks, publish native pipeline
tasks and pinned relationship definitions, and verify metadata by API.
Reconcile bot-preserved descriptions only after exact ownership checks.
Record the operator API-only rule and invented qualification/reset evidence.
</commit_message>
<xml_diff>
--- a/rules/sources/gleif/MAPPING.xlsx
+++ b/rules/sources/gleif/MAPPING.xlsx
@@ -13,7 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critical data elements" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data quality" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Who wins" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline targets" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline steps" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2469,6 +2471,402 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Run checks</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Lease seconds</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Heartbeat seconds</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Rules path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>manifest.hash, work.accounting, journal.delivered</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>umbrellas</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>manifest.hash, work.accounting, journal.delivered</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.umbrellas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Operation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Requires</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Leases</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Checks</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Rules path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>source.read</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, source.output</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering.steps[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>prepare</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>mdm.prepare</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, mdm.prepared</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering.steps[1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>mdm.merge</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>prepare</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>{batch_id}</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>mdm:consumer:{consumer}</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, mdm.committed</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering.steps[2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>journal.record</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, journal.recorded</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering.steps[3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>umbrellas</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>pairs</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>source.read</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, source.output</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.umbrellas.steps[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>umbrellas</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>journal.record</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>pairs</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, journal.recorded</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.umbrellas.steps[1]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Catalog every configured entity and pipeline with API verification (#1242)
* Cover configured entities and pipelines in the rules catalog

Generate all source/pipeline/relationship workbooks, publish native pipeline
tasks and pinned relationship definitions, and verify metadata by API.
Reconcile bot-preserved descriptions only after exact ownership checks.
Record the operator API-only rule and invented qualification/reset evidence.

* Qualify installed catalog commands and bundled mapping documents

---------

Co-authored-by: Aneena Ananth <aneenaananth@MacBook-Pro.local>
</commit_message>
<xml_diff>
--- a/rules/sources/gleif/MAPPING.xlsx
+++ b/rules/sources/gleif/MAPPING.xlsx
@@ -13,7 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critical data elements" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data quality" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Who wins" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline targets" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline steps" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2469,6 +2471,402 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Run checks</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Lease seconds</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Heartbeat seconds</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Rules path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>manifest.hash, work.accounting, journal.delivered</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>umbrellas</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>manifest.hash, work.accounting, journal.delivered</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.umbrellas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Operation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Requires</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Leases</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Checks</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Rules path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>source.read</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, source.output</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering.steps[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>prepare</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>mdm.prepare</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, mdm.prepared</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering.steps[1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>mdm.merge</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>prepare</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>{batch_id}</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>mdm:consumer:{consumer}</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, mdm.committed</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering.steps[2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>mastering</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>journal.record</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, journal.recorded</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.mastering.steps[3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>umbrellas</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>pairs</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>source.read</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, source.output</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.umbrellas.steps[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>umbrellas</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>journal.record</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>pairs</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>{unit}</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>artifact:{destination}</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>input.hash, output.receipt, journal.recorded</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>bookkeeping.targets.umbrellas.steps[1]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>